<commit_message>
Add DESeq2/tximport Salmon analysis script
Add a new R script (DESeq2_salmone_L1_L24.R) implementing a full tximport + DESeq2 pipeline for the LjFUN L1-L24 timecourse. The script loads Salmon quantifications, builds tx2gene from transcript FASTA/annotations, exports raw counts/TPM/normalized counts, runs VST/PCA, performs multiple contrasts with lfcShrink (ashr), writes MA plots and DEG tables, and generates DEG summary barplots and Venn diagrams. Also update the example Sample Register.xlsx used as metadata. Intended to provide end-to-end processing and summary outputs for the ljfun vs WT +/- N timecourse.
</commit_message>
<xml_diff>
--- a/Bulk RNA-seq/Salmon/ExampleData/Copy of Sample Register.xlsx
+++ b/Bulk RNA-seq/Salmon/ExampleData/Copy of Sample Register.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\LAB - OPV - Dugald_Reid\Genomics\RNAseq datasets\220126 cowpea lotus faba Novogene\X201SC25100870-Z01-F001\01.RawData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://latrobeuni-my.sharepoint.com/personal/bweeyang_ltu_edu_au/Documents/Documents/GitHub/Reid-Smith-Lab/Bulk RNA-seq/Salmon/ExampleData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39F8CB7D-7596-467B-A3C3-10931B84DA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{39F8CB7D-7596-467B-A3C3-10931B84DA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8396FCD8-4F88-4C9B-8AC2-A652D2C25874}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-255" windowWidth="29040" windowHeight="15720" xr2:uid="{78418E0A-BB8A-41CC-973A-0E04FCCE5F8E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{78418E0A-BB8A-41CC-973A-0E04FCCE5F8E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -973,18 +973,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E2FF8F8-35B4-4542-B1A0-754F8B41B2E3}">
-  <dimension ref="A1:H89"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J89"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" customWidth="1"/>
-    <col min="6" max="6" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" customWidth="1"/>
+    <col min="3" max="3" width="19.109375" customWidth="1"/>
+    <col min="4" max="4" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.88671875" customWidth="1"/>
+    <col min="6" max="6" width="29.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>58</v>
       </c>
@@ -1010,7 +1010,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>59</v>
       </c>
@@ -1036,7 +1036,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>59</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>59</v>
       </c>
@@ -1114,7 +1114,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>59</v>
       </c>
@@ -1140,7 +1140,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>59</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>59</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>59</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1244,7 +1244,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>59</v>
       </c>
@@ -1270,7 +1270,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -1296,7 +1296,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>59</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>59</v>
       </c>
@@ -1348,7 +1348,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>59</v>
       </c>
@@ -1374,7 +1374,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>59</v>
       </c>
@@ -1400,7 +1400,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>59</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>59</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>59</v>
       </c>
@@ -1478,7 +1478,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>59</v>
       </c>
@@ -1504,7 +1504,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>59</v>
       </c>
@@ -1530,7 +1530,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -1556,7 +1556,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>59</v>
       </c>
@@ -1582,7 +1582,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>59</v>
       </c>
@@ -1608,7 +1608,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>59</v>
       </c>
@@ -1634,7 +1634,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>59</v>
       </c>
@@ -1660,7 +1660,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>59</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -1738,7 +1738,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>127</v>
       </c>
@@ -1764,7 +1764,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>127</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>127</v>
       </c>
@@ -1816,7 +1816,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>127</v>
       </c>
@@ -1842,7 +1842,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>127</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>127</v>
       </c>
@@ -1894,7 +1894,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>127</v>
       </c>
@@ -1920,7 +1920,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>127</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>127</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>127</v>
       </c>
@@ -1998,7 +1998,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>127</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>127</v>
       </c>
@@ -2050,7 +2050,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>127</v>
       </c>
@@ -2076,7 +2076,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>127</v>
       </c>
@@ -2102,7 +2102,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>127</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>127</v>
       </c>
@@ -2154,7 +2154,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>127</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>127</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>127</v>
       </c>
@@ -2232,7 +2232,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>127</v>
       </c>
@@ -2258,7 +2258,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>127</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>127</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>127</v>
       </c>
@@ -2336,7 +2336,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>127</v>
       </c>
@@ -2362,7 +2362,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>128</v>
       </c>
@@ -2388,7 +2388,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>128</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>128</v>
       </c>
@@ -2440,7 +2440,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>128</v>
       </c>
@@ -2466,7 +2466,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>128</v>
       </c>
@@ -2492,7 +2492,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>128</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>128</v>
       </c>
@@ -2544,7 +2544,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>128</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>128</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>128</v>
       </c>
@@ -2622,7 +2622,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>128</v>
       </c>
@@ -2648,7 +2648,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>128</v>
       </c>
@@ -2674,7 +2674,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>128</v>
       </c>
@@ -2700,7 +2700,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>128</v>
       </c>
@@ -2726,7 +2726,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>128</v>
       </c>
@@ -2752,7 +2752,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>128</v>
       </c>
@@ -2778,7 +2778,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>128</v>
       </c>
@@ -2804,7 +2804,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>128</v>
       </c>
@@ -2830,7 +2830,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>128</v>
       </c>
@@ -2856,7 +2856,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>128</v>
       </c>
@@ -2882,7 +2882,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>128</v>
       </c>
@@ -2908,7 +2908,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>128</v>
       </c>
@@ -2934,7 +2934,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>128</v>
       </c>
@@ -2960,7 +2960,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>128</v>
       </c>
@@ -2986,7 +2986,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>166</v>
       </c>
@@ -3012,7 +3012,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>166</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>166</v>
       </c>
@@ -3064,7 +3064,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>166</v>
       </c>
@@ -3090,7 +3090,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>166</v>
       </c>
@@ -3116,7 +3116,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>166</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>166</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>166</v>
       </c>
@@ -3193,8 +3193,12 @@
       <c r="H85">
         <v>29</v>
       </c>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J85">
+        <f>29/7</f>
+        <v>4.1428571428571432</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>166</v>
       </c>
@@ -3220,7 +3224,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>166</v>
       </c>
@@ -3246,7 +3250,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>166</v>
       </c>
@@ -3272,7 +3276,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>166</v>
       </c>
@@ -3303,4 +3307,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{9aee26d8-97c2-4fad-8900-96735f6dc73f}" enabled="0" method="" siteId="{9aee26d8-97c2-4fad-8900-96735f6dc73f}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>